<commit_message>
Update upcoming events layout, data, and header styling
</commit_message>
<xml_diff>
--- a/src/events/Nova Stella Events.xlsx
+++ b/src/events/Nova Stella Events.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emmalufox/Code/Nova Stella/nova-stella/src/events/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A77F062-C8A3-BC46-A450-2B76A820BE21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DDB63D9-5F64-8B46-9E85-F5921E4C7159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17440" xr2:uid="{6E1F4C7A-1D7E-924D-9EE1-8636AFCD4F36}"/>
   </bookViews>
@@ -608,7 +608,7 @@
     <tableColumn id="9" xr3:uid="{212AF97D-2057-7D43-88D9-E0CE3C1634B0}" name="Speaker Website" dataDxfId="7"/>
     <tableColumn id="10" xr3:uid="{BC08696A-9796-EA4C-AE48-D871B744D793}" name="Talk Title" dataDxfId="6"/>
     <tableColumn id="11" xr3:uid="{AE0CCD02-01F4-E941-A639-F020519757FB}" name="Talk Blurb" dataDxfId="5">
-      <calculatedColumnFormula>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</calculatedColumnFormula>
+      <calculatedColumnFormula>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="12" xr3:uid="{C9CC2950-352B-8E4F-B8E2-418A618ECF42}" name="Online Eventbrite Link" dataDxfId="4" dataCellStyle="Hyperlink"/>
     <tableColumn id="13" xr3:uid="{53430355-0298-ED40-BD24-1289A5FB979E}" name="In Person Eventbrite Link" dataDxfId="3" dataCellStyle="Hyperlink"/>
@@ -1064,7 +1064,7 @@
         <v>11</v>
       </c>
       <c r="N2" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
         <v>Join us at Nova Stella for a mystical journey into Grandmother Winter's House of Healing : A Trance Journey for Witches
 We are absolutely delighted and thrilled to be able to say that our first speaker of 2026 on Monday the 26th January at the Angel Pub in Shoreditch will be none other than Sara Mastros. The talk will be on: "Grandmother Winter's House of Healing: A Trance Journey for Witches".
 Sara L. Mastros is the author of “Introduction to Witchcraft: Thirteen Lessons in the Practice of Magic," The Sorcery of Solomon: A Guide to the 44 Planetary Pentacles of the Magician King", “The Big Book of Magical Incense", and "Orphic Hymns Grimoire.”
@@ -1123,8 +1123,8 @@
         <v>29</v>
       </c>
       <c r="N3" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by Professor Ronald Hutton in convivial company.
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Professor Ronald Hutton in convivial company.
 Highly regarded by our community, Ronald Hutton is Professor of History at the University of Bristol, the Gresham Professor of Divinity at London, and a Fellow of the Royal Historical Society, the Society of Antiquaries, the Learned Society of Wales, and the British Academy. He has held a number of public posts and been appointed a Commander of the Order of the British Empire. He is currently the chair of the first national Blue Plaques Panel. He has published nineteen books and ninety-six essays on a wide range of subjects including British history between 1400 and 1700, ancient and modern paganism in Britain, the British ritual year, and Siberian shamanism.</v>
       </c>
       <c r="O3" s="10" t="s">
@@ -1177,7 +1177,7 @@
         <v>51</v>
       </c>
       <c r="N4" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
         <v>Chaos Magick stands at the limits of both left and right factions of magick, as well as extremes of gender, sexual, traditional, and radical ideology. This talk will dispute the false perception of chaos magick as belonging to certain kinds of magi, celebrating the role of art, experimentation, and non-traditional magical rites currently celebrated in queer chaos. Using all modes of art and imagination, the talk will show that chaos magick is ultimately for the dissolution of self and the evolution of becoming—against the ascension of being—and can offer liberation toward radical cosmic and ecological futures.
 Patricia is a researcher who has published in the areas of continental philosophy (especially Deleuze, Guattari, Serres, Irigaray, Lyotard, Kristeva, Blanchot, Ranciere), feminism, queer theory, posthuman theory, horror film, body modification, animal rights/abolitionism, cinesexuality, ethics and death studies.
 Patricia MacCormack is Professor of Continental Philosophy. She is the author of Cinesexuality (Routledge 2008) and Posthuman Ethics (Routledge 2012) and the editor of The Animal Catalyst (Bloomsbury 2014), Deleuze and the Animal (EUP 2017), Deleuze and the Schizoanalysis of Cinema (Continuum 2008) and Ecosophical Aesthetics (Bloomsbury 2018). Her newest book is The Ahuman Manifesto: Activisms for the End of the Anthropocene. She recently completed a Leverhulme Fellow researching and developing Death Activism and completing the monograph Death Activism for Bloomsbury. She is also the author of numerus journal articles and anthology chapters.
@@ -1238,8 +1238,8 @@
         <v>47</v>
       </c>
       <c r="N5" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by John Callow in convivial company.
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by John Callow in convivial company.
 John Callow is an author, historian and trade unionist.
 He has written widely on Early Modern witchcraft, politics and popular culture. His books include Witchcraft &amp; Magic in Sixteenth- and Seventeenth-Century Europe (co-authored with Professor Geoffrey Scarre); James II: King in Exile; Embracing the Darkness: A Cultural History of Witchcraft, and The Last Witches of England: A Tragedy of Sorcery and Superstition. 
 He has appeared on the BBC’s The One Show to discuss the roots of Hallowe’en; on the BBC Radio 4 documentary, It Must be Witchcraft;  Find My Past's The Great Fire of London; and the Discovery Channel's four-part series, The Salem Witches. He has also appeared regularly on the History Hit podcast series.</v>
@@ -1292,8 +1292,8 @@
         <v>47</v>
       </c>
       <c r="N6" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by Sara Hannant in convivial company.
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Sara Hannant in convivial company.
 Sara Hannant’s photographic practice is inspired by witchcraft, magic, and folklore. She is fascinated by the diverse expressive qualities of photography and uses analogue, digital, and alternative processes.
 Her latest work Panic:Visions of The Horned God in the English Country Garden will be exhibited at State 51 as part of Photomonth festival in London. A book featuring Sara Hannant’s photographs and texts by Simon Coston, Sara Hannant and Ronald Hutton, will be available from Strange Attractor Press in Spring 2026.
 Recent award-winning work includes Anima (2023), Dark Solace (2022) and Force Fields (2021), which investigate the enchanted materiality of found magic lantern slides. Her series Betwixt, selected by Alice Gabriner for Best in Show, International Photography Award (2021) depicts children interacting with imaginary photographic worlds.
@@ -1350,8 +1350,8 @@
         <v>47</v>
       </c>
       <c r="N7" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by Meggie Reid in convivial company.
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Meggie Reid in convivial company.
 Meg is a a witch, pagan, intuitive Tarot reader, Rune reader, Seidr practitioner, energy healer, singer/songwriter and bellydancer, who considers it her mission to provide insight and guidance to those who seek it._x000B_It is one of her great passions in life to be able to offer service to the world and all who need it, with an emphasis on authenticity, empathy, embodiment and understanding. Meg has trained alongside Magin Rose, Katie Gerrard, Andre Henriques and Dance Body Mind._x000B_She believes that all our paths are unique and important and it’s integral to me that everyone discovers their own vital piece in our cosmic puzzle.</v>
       </c>
       <c r="O7" s="10"/>
@@ -1400,8 +1400,8 @@
         <v>47</v>
       </c>
       <c r="N8" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by Caroline Wise in convivial company.
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Caroline Wise in convivial company.
 Caroline Wise compiled the book Finding Elen, the Quest for Elen of the Ways, which seeks out the antlered goddess. Caroline is an ordained priestess of the Goddess, and has contributed to several books on goddesses, on woman magical pioneers, and on Mythic London. Caroline trains women to become priestesses and oracles of the goddess. She had led workshops and talks based on these subjects in UK, Italy, USA and Germany, and she organised Goddess conferences in the London from 1990.</v>
       </c>
       <c r="O8" s="10"/>
@@ -1452,7 +1452,7 @@
         <v>81</v>
       </c>
       <c r="N9" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
         <v>This talk will look at loss, and how people attempt to reconnect with loved ones who have passed, via AI, VR, hallucinogenics and such, and reflect on these experiences. Rebecca Lambert is an archaeologist dedicated to public engagement, accessibility, and innovative research practices. Her approach sits at the intersection of prehistory, art history, architectural history and design, and mixed-media creative practice, which she explores through the lenses of space, place, temporality, and connection.
 Rebecca’s previous research has been critically received, with the Underpasses Are Liminal Places project having been cited as ‘a significant innovation in public archaeology.’ Rebecca has also contributed extensively to journals and publications, exploring topics such as subterranean archaeology, psychogeography, and the intersection of archaeology and art.
 Her research also features in academic and non-fiction texts, including Teaching and Learning the Archaeology of the Contemporary Era (Moshenska (Ed), 2024; and Fiona Robertson’s Stone Lands: A Journey of Darkness and Light (2025), a Times’ Book of the Year.
@@ -1509,8 +1509,8 @@
         <v>47</v>
       </c>
       <c r="N10" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by Jason Atomic in convivial company.
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Jason Atomic in convivial company.
 From London to Tokyo, New York or Berlin Jason Atomic is a familiar face in a variety of subcultures.
 Despite a background in comix he discovered real life to be more interesting than fiction and began a documenting the freak icons of the underground art, music and club scenes in his colourful energetic paintings and sketchbooks.
 Says Atomic:
@@ -1565,8 +1565,8 @@
         <v>47</v>
       </c>
       <c r="N11" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by Ruth Bayer in convivial company.
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Ruth Bayer in convivial company.
 Born in Salzburg, Austria, Ruth grew up with the tales and sagas of the surrounding mountains and she has always been particularly fascinated by the myths and legends of goddesses and gods . Her photography has been widely published, including two books with Strange Attractor Press including her work with the band Coil. In collaboration with Caroline Wise she has produced two books – Here Comes The Candle; a Summoning of London Ghosts, and a forthcoming work on Mystical London. Ruth is High Priestess of a known North London Gardnerian Coven.</v>
       </c>
       <c r="O11" s="10"/>
@@ -1615,8 +1615,8 @@
         <v>47</v>
       </c>
       <c r="N12" s="8" t="str">
-        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
-        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enligtening talk by Paul Bland in convivial company.
+        <f>IF(Events[[#This Row],[Speaker]]="TBC","",IF(ISBLANK(Events[[#This Row],[Talk Blurb Text]]),_xlfn.CONCAT("Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by ",Events[[#This Row],[Speaker]]," in convivial company.",CHAR(10),Events[[#This Row],[Speaker Bio]]),Events[[#This Row],[Talk Blurb Text]]))</f>
+        <v>Join us at the top floor of the Angel Pub in Shoreditch for an enlightening talk by Paul Bland in convivial company.
 Paul is a London born 2nd degree witch in a Hackney coven. He has developed a Moon curriculum for his coven. In the mundane world he teaches and practices diagnostic imaging in healthcare.</v>
       </c>
       <c r="O12" s="10"/>

</xml_diff>